<commit_message>
Replace price tiers with concrete prices
Replace the abstract "價格帶" (low/medium/high CP) attribute with explicit price levels for each market: "售價(USD)" ($19.99/$34.99/$59.99) for the US and "售價(JPY)" (¥2,999/¥4,999/¥7,999) for Japan. Updated generate_product_cards.py to use the new attribute names/values and adjusted markdown generation accordingly; regenerated output_conjoint/product_cards.xlsx and output_conjoint/product_cards_report.md to reflect the concrete prices in product cards and level balance tables.
</commit_message>
<xml_diff>
--- a/output_conjoint/product_cards.xlsx
+++ b/output_conjoint/product_cards.xlsx
@@ -442,7 +442,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(USD)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(JPY)</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2309,7 +2309,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2403,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
     </row>
@@ -2685,7 +2685,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
     </row>
@@ -2952,12 +2952,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(USD)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>$19.99</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -2967,12 +2967,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(USD)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>$34.99</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -2982,12 +2982,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(USD)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>$59.99</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3523,12 +3523,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(JPY)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>低CP值</t>
+          <t>¥2,999</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3538,12 +3538,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(JPY)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>中CP值</t>
+          <t>¥4,999</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3553,12 +3553,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>價格帶</t>
+          <t>售價(JPY)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>高CP值</t>
+          <t>¥7,999</t>
         </is>
       </c>
       <c r="C25" t="n">

</xml_diff>